<commit_message>
Correction mauvais usage de la fusion de JDV (#61)
* remplace valueset addings by TRE

* fix syntax error ae743435e3da4eab5db064d1e999099cc1f7cc39
</commit_message>
<xml_diff>
--- a/ig/main/ValueSet-method-glucose-vs.xlsx
+++ b/ig/main/ValueSet-method-glucose-vs.xlsx
@@ -7,14 +7,14 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
-    <sheet name="Include ValueSets" r:id="rId4" sheetId="2"/>
-    <sheet name="Include ValueSets 2" r:id="rId5" sheetId="3"/>
+    <sheet name="Include from TRE-R312-LPP" r:id="rId4" sheetId="2"/>
+    <sheet name="Include from TRE-R307-NCIT" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t>Property</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-09-19T16:09:26+00:00</t>
+    <t>2023-09-19T16:18:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -91,13 +91,22 @@
     <t>BooleanType[null]</t>
   </si>
   <si>
-    <t>ValueSet URL</t>
-  </si>
-  <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J155-MethodGlucoseSanguin-ENS/FHIR/JDV-J155-MethodGlucoseSanguin-ENS</t>
-  </si>
-  <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J156-MethodGlucoseInterstitiel-ENS/FHIR/JDV-J156-MethodGlucoseInterstitiel-ENS</t>
+    <t>Codes</t>
+  </si>
+  <si>
+    <t>All codes</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>System URI</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/TRE_R312-LPP/FHIR/TRE-R312-LPP</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/TRE_R307-NCIT/FHIR/TRE-R307-NCIT</t>
   </si>
 </sst>
 </file>
@@ -351,7 +360,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.703125" customWidth="true"/>
@@ -368,6 +377,22 @@
         <v>26</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -375,7 +400,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.703125" customWidth="true"/>
@@ -389,7 +414,23 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
         <v>27</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>